<commit_message>
feat: confirmación en acciones destructivas + debounce en búsqueda de maestra
- ConfirmDialog reutilizable con hook useConfirmDialog (IsDangerous, botón rojo)
- HoldingsPage: confirmación antes de eliminar RUTs, dominios y reglas avanzadas
- useDebounce hook (300ms) aplicado en búsqueda de itemcode en OcDetailPanel
- Fix TypeScript: confirm prop propagado hasta RuleEditor

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HOMO INDISA.xlsx
+++ b/HOMO INDISA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agsvsai-my.sharepoint.com/personal/samuel_belmar_nemochile_cl/Documents/Escritorio/PROYECTOS/INGRESO OC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B505C22-8EC7-49F4-9956-DA6D34352120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{6B505C22-8EC7-49F4-9956-DA6D34352120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F95FF23A-B92D-4EAF-A8A6-B3EF48DFF1A1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{686751A4-5191-43E7-BADF-4E266E1A45AB}"/>
+    <workbookView xWindow="28680" yWindow="870" windowWidth="29040" windowHeight="15720" xr2:uid="{686751A4-5191-43E7-BADF-4E266E1A45AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>COD CLINICA</t>
   </si>
@@ -153,6 +153,12 @@
   </si>
   <si>
     <t>TAP00001</t>
+  </si>
+  <si>
+    <t>KNE00110</t>
+  </si>
+  <si>
+    <t>BANDEJA C18 ESTERIL</t>
   </si>
 </sst>
 </file>
@@ -525,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E2C92E4-877E-4FD9-AC11-7C26B73DB56D}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
@@ -876,6 +882,20 @@
         <v>4026</v>
       </c>
     </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>22200082</v>
+      </c>
+      <c r="B18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18">
+        <v>455</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F17" xr:uid="{2E2C92E4-877E-4FD9-AC11-7C26B73DB56D}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F17">

</xml_diff>